<commit_message>
feature/fsel-5228: update api import and export student by admin school
</commit_message>
<xml_diff>
--- a/Services/Fsel.Identity/Fsel.Identity.Api/Resources/ExportExcelTemplates/Template_Export_Data_Student_By_Admin_School.xlsx
+++ b/Services/Fsel.Identity/Fsel.Identity.Api/Resources/ExportExcelTemplates/Template_Export_Data_Student_By_Admin_School.xlsx
@@ -5,12 +5,12 @@
   <workbookPr showInkAnnotation="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\fsel_src\Services\Fsel.Identity\Fsel.Identity.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{258A80AC-31EC-417F-8E23-BE8D565599AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE48524-0518-45C8-81C4-8E0EB231C9BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Full Name
 (Họ và tên)</t>
@@ -46,12 +46,16 @@
 (Tên đăng nhập)</t>
   </si>
   <si>
-    <t>Password
-(Mật khẩu)</t>
-  </si>
-  <si>
     <t>Grade
 (Khối học)</t>
+  </si>
+  <si>
+    <t>Password
+(Mật khẩu tạm thời)</t>
+  </si>
+  <si>
+    <t>Created Date
+(Ngày tạo)</t>
   </si>
 </sst>
 </file>
@@ -110,16 +114,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -446,44 +447,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="39" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.7109375" style="6" customWidth="1"/>
-    <col min="5" max="5" width="18.42578125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="20.85546875" style="6" customWidth="1"/>
-    <col min="7" max="7" width="46.140625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" style="9" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="2"/>
+    <col min="4" max="4" width="19.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="20.85546875" style="5" customWidth="1"/>
+    <col min="7" max="7" width="46.140625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="18.28515625" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="7" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:9" s="6" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>6</v>
+      <c r="I1" s="7" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>